<commit_message>
Simplify rules workbook to a single sheet, no template scaffolding
</commit_message>
<xml_diff>
--- a/DS-Project-QC-Regras.xlsx
+++ b/DS-Project-QC-Regras.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Regras Ativas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Novas Regras" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Regras" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,12 +33,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="0066746F"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
@@ -48,13 +41,8 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -74,21 +62,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FAF0DC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7E7E4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFDE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,31 +91,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,12 +474,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -525,47 +490,60 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>O que o motor verifica hoje em cada Project Package carregado.</t>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Regra</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>O que verifica</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Regra</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>O que verifica</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="A4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Typos sistêmicos</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Erros de digitação conhecidos (ex.: "LENGHT" em vez de "LENGTH") que se repetem pelo pacote inteiro — sinalizado como uma correção só ("corrigir em todo lugar"), não um achado por prancha.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Ativa</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
+      <c r="A5" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Typos sistêmicos</t>
+          <t>Código duplicado em schedule/legenda</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Erros de digitação conhecidos (ex.: "LENGHT" em vez de "LENGTH") que se repetem pelo pacote inteiro — sinalizado como uma correção só ("corrigir em todo lugar"), não um achado por prancha.</t>
+          <t>Um mesmo código (ex.: "D2", "CE04") aparecendo em mais de uma linha distinta dentro da mesma tabela — deixa ambíguo qual linha um callout na planta está referenciando.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -575,17 +553,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>2</v>
+      <c r="A6" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Código duplicado em schedule/legenda</t>
+          <t>Quantidade placeholder</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Um mesmo código (ex.: "D2", "CE04") aparecendo em mais de uma linha distinta dentro da mesma tabela — deixa ambíguo qual linha um callout na planta está referenciando.</t>
+          <t>Quantidade do tipo "XX SQFT" deixada sem preencher em schedule/legenda.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -595,17 +573,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>3</v>
+      <c r="A7" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Quantidade placeholder</t>
+          <t>Clearance de porta</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Quantidade do tipo "XX SQFT" deixada sem preencher em schedule/legenda.</t>
+          <t>Porta de passagem (swing/pocket) abaixo da largura mínima de código: 34" pra swing, 32" pra pocket. Só verifica tipos claramente de passagem (SWING, DOUBLE, INVISIBLE, POCKET).</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -615,17 +593,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>4</v>
+      <c r="A8" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Clearance de porta</t>
+          <t>Sequência de revisão</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Porta de passagem (swing/pocket) abaixo da largura mínima de código: 34" pra swing, 32" pra pocket. Só verifica tipos claramente de passagem (SWING, DOUBLE, INVISIBLE, POCKET).</t>
+          <t>Duas checagens no quadro de revisão de cada prancha: (a) os números de revisão precisam ser uma sequência sem buraco; (b) a data de uma revisão não pode ser anterior à da revisão de antes.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -635,17 +613,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>5</v>
+      <c r="A9" s="3" t="n">
+        <v>6</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Sequência de revisão</t>
+          <t>Cota não resolvida (TBD) em demolição/construção/reforço</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Duas checagens no quadro de revisão de cada prancha: (a) os números de revisão precisam ser uma sequência sem buraco; (b) a data de uma revisão não pode ser anterior à da revisão de antes.</t>
+          <t>Nota de demolição, construção ou reforço que usa uma dessas palavras-chave mas deixa a cota como "TBD" em vez de um número resolvido.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -655,17 +633,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
+      <c r="A10" s="3" t="n">
+        <v>7</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Cota não resolvida (TBD) em demolição/construção/reforço</t>
+          <t>Altura de teto (código x Ceiling Schedule)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Nota de demolição, construção ou reforço que usa uma dessas palavras-chave mas deixa a cota como "TBD" em vez de um número resolvido.</t>
+          <t>O código de teto carimbado na planta (ex.: "CE04" sobre "132\" A.F.F.") precisa bater com a altura da mesma linha de código no Ceiling Schedule.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -675,17 +653,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
+      <c r="A11" s="3" t="n">
+        <v>8</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Altura de teto (código x Ceiling Schedule)</t>
+          <t>Quantidade de luminária (só pacotes Revit)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>O código de teto carimbado na planta (ex.: "CE04" sobre "132\" A.F.F.") precisa bater com a altura da mesma linha de código no Ceiling Schedule.</t>
+          <t>Quantas vezes um código de luminária aparece de fato no RCP/Lighting/Circuits comparado com a quantidade do Fixture Schedule. Só funciona em pacotes Revit — AutoCAD não tagueia cada luminária individualmente.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -695,256 +673,28 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>8</v>
+      <c r="A12" s="3" t="n">
+        <v>9</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Quantidade de luminária (só pacotes Revit)</t>
+          <t>Especificação não resolvida (TBD)</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Quantas vezes um código de luminária aparece de fato no RCP/Lighting/Circuits comparado com a quantidade do Fixture Schedule. Só funciona em pacotes Revit — AutoCAD não tagueia cada luminária individualmente.</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Ativa</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Especificação não resolvida (TBD)</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
           <t>Uma célula de schedule/legenda com o valor de acabamento/material deixado só como "TBD". Desligada por padrão (TBD é normal em early stage) — marque "Verificar specs TBD" ao anexar o PDF na timeline do projeto pra ligar.</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>Opcional</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Regras removidas (testadas e descartadas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Regra</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Motivo da remoção</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Spec de porta incompleta</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Flagava colunas em branco no Door Schedule (modelo, room, acabamento, hardware, sentido de abertura) — removida porque às vezes a spec realmente ainda não existe, e virava ruído.</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Removida</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A15:D15"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Novas regras propostas</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Preencha uma linha por regra nova e me carregue este arquivo — eu implemento e devolvo marcado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Legenda: preencha só as células brancas (colunas A a D). A linha amarela é um exemplo — pode apagar ou sobrescrever.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Nome da regra</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>O que verificar</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Onde já vi isso dar problema (prancha/projeto real)</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Exceção conhecida</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Nichos com tamanho errado</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Nicho de banheiro/closet cotado na planta de Construção precisa bater com o tamanho real do file seam usado no Shop Drawing — hoje só é cotado no SD.</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Hibiscus Res, rodada NEW (#15)</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Nenhuma conhecida ainda</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Proposta</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="10" t="inlineStr"/>
-      <c r="D8" s="10" t="inlineStr"/>
-      <c r="E8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="10" t="inlineStr"/>
-      <c r="E9" s="10" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="10" t="inlineStr"/>
-      <c r="D10" s="10" t="inlineStr"/>
-      <c r="E10" s="10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="10" t="inlineStr"/>
-      <c r="D11" s="10" t="inlineStr"/>
-      <c r="E11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="10" t="inlineStr"/>
-      <c r="D12" s="10" t="inlineStr"/>
-      <c r="E12" s="10" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="10" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr"/>
-      <c r="E13" s="10" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="10" t="inlineStr"/>
-      <c r="D14" s="10" t="inlineStr"/>
-      <c r="E14" s="10" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="10" t="inlineStr"/>
-      <c r="D15" s="10" t="inlineStr"/>
-      <c r="E15" s="10" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A4:E4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Track proposed cross-sheet dimension-consistency rule as pending
</commit_message>
<xml_diff>
--- a/DS-Project-QC-Regras.xlsx
+++ b/DS-Project-QC-Regras.xlsx
@@ -42,7 +42,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +62,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FAF0DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -107,6 +112,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -692,6 +700,26 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Cota consistente entre pranchas</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>A mesma cota de um elemento (ex.: cota de um curtain pocket) precisa bater em todas as pranchas onde aparece. Confirmado nos dados reais (CASA@63 R04) que a posição na página varia entre disciplinas (Construction vs Ceiling vs Lighting), então não dá pra linkar só por posição — precisa de um exemplo real de conflito pra calibrar sem gerar falso positivo.</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Pendente — aguardando exemplo real</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>